<commit_message>
feat: data auto fill
</commit_message>
<xml_diff>
--- a/Student_Management_Flask/data/students.xlsx
+++ b/Student_Management_Flask/data/students.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,6 +455,86 @@
       <c r="D2" t="inlineStr">
         <is>
           <t>CSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2024-miit-cse-050</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Zaw Zaw Aung</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2025-miit-cse-029</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Hlaing Myo Aung</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2025-miit-cse-060</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Oak Kar Aung</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2025-miit-ece-041</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Htet Aung Win</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ECE</t>
         </is>
       </c>
     </row>

</xml_diff>